<commit_message>
COde committed for second testcase
</commit_message>
<xml_diff>
--- a/src/test/resources/com/ab/excel/TestData.xlsx
+++ b/src/test/resources/com/ab/excel/TestData.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="9">
   <si>
     <t>Username</t>
   </si>
@@ -30,12 +30,6 @@
     <t>Pass@Pass@123</t>
   </si>
   <si>
-    <t>new.user2@test.tina5s.com</t>
-  </si>
-  <si>
-    <t>Qisw*H01%$%4</t>
-  </si>
-  <si>
     <t>Runmode</t>
   </si>
   <si>
@@ -45,17 +39,17 @@
     <t>LoginTest</t>
   </si>
   <si>
-    <t>LoginTest1</t>
-  </si>
-  <si>
     <t>zz@test.tina5s.com</t>
+  </si>
+  <si>
+    <t>New_Record</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -70,6 +64,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF1290C3"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -93,9 +93,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -398,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31" bestFit="1" customWidth="1"/>
@@ -407,7 +408,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -418,7 +419,7 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -429,23 +430,23 @@
         <v>3</v>
       </c>
       <c r="C3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>3</v>
       </c>
       <c r="C4" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>9</v>
+      <c r="A6" s="2" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -456,7 +457,7 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -467,29 +468,7 @@
         <v>3</v>
       </c>
       <c r="C8" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>4</v>
-      </c>
-      <c r="B9" t="s">
         <v>5</v>
-      </c>
-      <c r="C9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>2</v>
-      </c>
-      <c r="B10" t="s">
-        <v>3</v>
-      </c>
-      <c r="C10" t="s">
-        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -497,6 +476,7 @@
     <hyperlink ref="B4" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>